<commit_message>
Verifica settimanale (parziale): deduplica cross-file su tutti i file /output
Marcati 202 nuovi duplicati (su 216 totali rilevati globalmente, 14 già
marcati da run precedenti) in 41 file .xlsx, annotando il campo note con
riferimento al file canonico (occorrenza più vecchia). Nessuna riga
cancellata, nessuna colonna modificata oltre a note/stato_verifica.

Il doppio controllo AI (upgrade stato_verifica) sui file nuovi di questo
run è in corso in background; seguirà un commit successivo con i risultati
e l'aggiornamento di weekly_verify_state.json / weekly_verify_log.md.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012RScj45V8Mb9fPDYDmrnEj
</commit_message>
<xml_diff>
--- a/output/2026-08-31_12_Italia_Toscana_Componentistica_Ventilazione_industriale.xlsx
+++ b/output/2026-08-31_12_Italia_Toscana_Componentistica_Ventilazione_industriale.xlsx
@@ -501,7 +501,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Attiva dal 1979, P.IVA 00267180974, sede Via dell'Agricoltura 27/29/31, Montemurlo (PO). Verificata tramite WebSearch (Kompass, misterimprese, sito ufficiale) - telefono confermato da fonte indipendente.</t>
+          <t>Attiva dal 1979, P.IVA 00267180974, sede Via dell'Agricoltura 27/29/31, Montemurlo (PO). Verificata tramite WebSearch (Kompass, misterimprese, sito ufficiale) - telefono confermato da fonte indipendente. [DUPLICATO — vedi anche: 2026-08-31_08_Italia_Toscana_Cleaning.xlsx]</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -536,10 +536,9 @@
           <t>055 898001</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>P.IVA 05792470485, fondata 2007/2008, 20-49 dipendenti. Telefono principale confermato; ulteriori numeri (055 898005 / 055 0941223) ed email non confermati da fonte indipendente - da ricontrollare. Possibile componente business anche HORECA.</t>
+          <t>P.IVA 05792470485, fondata 2007/2008, 20-49 dipendenti. Telefono principale confermato; ulteriori numeri (055 898005 / 055 0941223) ed email non confermati da fonte indipendente - da ricontrollare. Possibile componente business anche HORECA. [DUPLICATO — vedi anche: 2026-08-31_08_Italia_Toscana_Cleaning.xlsx]</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -581,7 +580,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Sede Via Trasimeno 3, Prato. Verificata tramite sito ufficiale e directory, forte coerenza col target.</t>
+          <t>Sede Via Trasimeno 3, Prato. Verificata tramite sito ufficiale e directory, forte coerenza col target. [DUPLICATO — vedi anche: 2026-08-31_08_Italia_Toscana_Cleaning.xlsx]</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -616,10 +615,9 @@
           <t>+39 0574 25801</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Sede Via per le Case Nuove 105, Prato; fondata 2005, 20-49 dipendenti. Telefono/email non confermati da fonte indipendente nei risultati - azienda e sito verificati.</t>
+          <t>Sede Via per le Case Nuove 105, Prato; fondata 2005, 20-49 dipendenti. Telefono/email non confermati da fonte indipendente nei risultati - azienda e sito verificati. [DUPLICATO — vedi anche: 2026-08-31_09_Italia_Toscana_Depolverazione_Trattamento_aria.xlsx]</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -738,7 +736,6 @@
           <t>+39 055 9155082</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>P.IVA 01805360482, attiva dal 1981. ATTENZIONE: fonti indicano attività anche su condizionamento/pompe di calore per uso residenziale - verificare la reale quota di business industriale.</t>
@@ -783,7 +780,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>P.IVA 01118460474, 10-19 dipendenti. Indirizzo e telefono confermati da fonte indipendente, coincidenti col dato grezzo.</t>
+          <t>P.IVA 01118460474, 10-19 dipendenti. Indirizzo e telefono confermati da fonte indipendente, coincidenti col dato grezzo. [DUPLICATO — vedi anche: 2026-08-31_08_Italia_Toscana_Cleaning.xlsx]</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">

</xml_diff>